<commit_message>
refactor: remove empty route nodes for readable projects
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M4原型.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M4原型.xlsx
@@ -197,7 +197,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -369,7 +369,7 @@
         </is>
       </c>
       <c r="C5" s="2">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -390,7 +390,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="10.0" customWidth="1"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">47 滨江国际社区</t>
+          <t xml:space="preserve">3 滨江国际社区</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -594,23 +594,23 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">河坊街铺</t>
+          <t xml:space="preserve">滨江国际社区</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">钱塘发展</t>
         </is>
       </c>
       <c r="F5" s="2">
-        <v>150</v>
+        <v>270</v>
       </c>
       <c r="G5" s="2">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 城市事件</t>
+          <t xml:space="preserve">4 河坊街铺</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -630,37 +630,33 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">河坊街铺</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">城市生活</t>
+        </is>
+      </c>
+      <c r="F6" s="2">
+        <v>150</v>
+      </c>
+      <c r="G6" s="2">
+        <v>36</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 南宋食坊</t>
+          <t xml:space="preserve">5 城市事件</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -675,33 +671,37 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">南宋食坊</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
-        </is>
-      </c>
-      <c r="F7" s="2">
-        <v>170</v>
-      </c>
-      <c r="G7" s="2">
-        <v>42</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">32 运河事件</t>
+          <t xml:space="preserve">6 南宋食坊</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -716,37 +716,33 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭城事件</t>
+          <t xml:space="preserve">南宋食坊</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">城市生活</t>
+        </is>
+      </c>
+      <c r="F8" s="2">
+        <v>170</v>
+      </c>
+      <c r="G8" s="2">
+        <v>42</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7 大莲花场馆</t>
+          <t xml:space="preserve">7 运河事件</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -761,33 +757,37 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">大莲花场馆</t>
+          <t xml:space="preserve">运河事件</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
-        </is>
-      </c>
-      <c r="F9" s="2">
-        <v>240</v>
-      </c>
-      <c r="G9" s="2">
-        <v>66</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 城市阳台</t>
+          <t xml:space="preserve">8 杭城事件</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -802,33 +802,37 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市阳台</t>
+          <t xml:space="preserve">杭城事件</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
-        </is>
-      </c>
-      <c r="F10" s="2">
-        <v>260</v>
-      </c>
-      <c r="G10" s="2">
-        <v>72</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">46 运河运动公园</t>
+          <t xml:space="preserve">9 大莲花场馆</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -843,37 +847,33 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘潮</t>
+          <t xml:space="preserve">大莲花场馆</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">钱塘发展</t>
+        </is>
+      </c>
+      <c r="F11" s="2">
+        <v>240</v>
+      </c>
+      <c r="G11" s="2">
+        <v>66</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10 地铁换乘</t>
+          <t xml:space="preserve">10 城市阳台</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -888,37 +888,33 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁换乘</t>
+          <t xml:space="preserve">城市阳台</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">钱塘发展</t>
+        </is>
+      </c>
+      <c r="F12" s="2">
+        <v>260</v>
+      </c>
+      <c r="G12" s="2">
+        <v>72</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 外环·钱塘线 / 37 地铁快线</t>
+          <t xml:space="preserve">11 运河运动公园</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -938,12 +934,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱江创意港</t>
+          <t xml:space="preserve">运河运动公园</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F13" s="2">
@@ -954,7 +950,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 创业事件</t>
+          <t xml:space="preserve">12 外环·钱塘线 / 31 地铁快线</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -974,37 +970,33 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">创业事件</t>
+          <t xml:space="preserve">钱江创意港</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">钱塘发展</t>
+        </is>
+      </c>
+      <c r="F14" s="2">
+        <v>230</v>
+      </c>
+      <c r="G14" s="2">
+        <v>62</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 未来创业营</t>
+          <t xml:space="preserve">13 创业事件</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1019,33 +1011,37 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">未来创业营</t>
+          <t xml:space="preserve">创业事件</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F15" s="2">
-        <v>300</v>
-      </c>
-      <c r="G15" s="2">
-        <v>90</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">14 项目验收</t>
+          <t xml:space="preserve">14 未来创业营</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1060,28 +1056,24 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">项目验收</t>
+          <t xml:space="preserve">未来创业营</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F16" s="2">
+        <v>300</v>
+      </c>
+      <c r="G16" s="2">
+        <v>90</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1090,7 +1082,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1118,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35 运河灯会</t>
+          <t xml:space="preserve">16 良渚陶艺村</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1167,7 +1159,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">17 城市公投</t>
+          <t xml:space="preserve">17 云栖工坊</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1187,37 +1179,33 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市公投</t>
+          <t xml:space="preserve">云栖工坊</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F19" s="2">
+        <v>250</v>
+      </c>
+      <c r="G19" s="2">
+        <v>68</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">18 云栖工坊</t>
+          <t xml:space="preserve">18 人才事件</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1232,33 +1220,37 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">云栖工坊</t>
+          <t xml:space="preserve">人才事件</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F20" s="2">
-        <v>250</v>
-      </c>
-      <c r="G20" s="2">
-        <v>68</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">19 人才事件</t>
+          <t xml:space="preserve">19 西溪营地</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1273,37 +1265,33 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">人才事件</t>
+          <t xml:space="preserve">西溪营地</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">生态文体</t>
+        </is>
+      </c>
+      <c r="F21" s="2">
+        <v>210</v>
+      </c>
+      <c r="G21" s="2">
+        <v>54</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20 西溪营地</t>
+          <t xml:space="preserve">20 运河夜游</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1323,23 +1311,23 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">西溪营地</t>
+          <t xml:space="preserve">运河夜游</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="F22" s="2">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="G22" s="2">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">21 城市公园</t>
+          <t xml:space="preserve">21 外环·运河线 / 27 水上巴士线</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1359,37 +1347,33 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市公园</t>
+          <t xml:space="preserve">武林夜市</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">城市生活</t>
+        </is>
+      </c>
+      <c r="F23" s="2">
+        <v>200</v>
+      </c>
+      <c r="G23" s="2">
+        <v>52</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 运河夜游</t>
+          <t xml:space="preserve">22 小河市集</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1409,23 +1393,23 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河夜游</t>
+          <t xml:space="preserve">小河市集</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="F24" s="2">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="G24" s="2">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">23 外环·运河线 / 28 水上巴士线</t>
+          <t xml:space="preserve">23 未来路演厅</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1450,23 +1434,23 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">武林夜市</t>
+          <t xml:space="preserve">未来路演厅</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="F25" s="2">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="G25" s="2">
-        <v>52</v>
+        <v>82</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">24 小河市集</t>
+          <t xml:space="preserve">24 桥西生活馆</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1491,7 +1475,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">小河市集</t>
+          <t xml:space="preserve">桥西生活馆</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1500,14 +1484,14 @@
         </is>
       </c>
       <c r="F26" s="2">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="G26" s="2">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">43 未来路演厅</t>
+          <t xml:space="preserve">25 地铁补给站</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1527,12 +1511,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">道具补给</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭城事件</t>
+          <t xml:space="preserve">地铁补给站</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1552,12 +1536,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">26 桥西生活馆</t>
+          <t xml:space="preserve">26 道具补给站</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
         </is>
       </c>
     </row>
@@ -1572,33 +1556,37 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">道具补给</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西生活馆</t>
+          <t xml:space="preserve">道具补给站</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
-        </is>
-      </c>
-      <c r="F28" s="2">
-        <v>190</v>
-      </c>
-      <c r="G28" s="2">
-        <v>50</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">42 地铁补给站</t>
+          <t xml:space="preserve">0 我的公寓</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
         </is>
       </c>
     </row>
@@ -1608,42 +1596,38 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">水上巴士内环</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给站</t>
+          <t xml:space="preserve">运河文创</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">生态文体</t>
+        </is>
+      </c>
+      <c r="F29" s="2">
+        <v>200</v>
+      </c>
+      <c r="G29" s="2">
+        <v>54</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 我的公寓</t>
+          <t xml:space="preserve">28 钱塘会展中心</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1658,37 +1642,33 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">武林门码头</t>
+          <t xml:space="preserve">钱塘会展中心</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">钱塘发展</t>
+        </is>
+      </c>
+      <c r="F30" s="2">
+        <v>280</v>
+      </c>
+      <c r="G30" s="2">
+        <v>78</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">29 运河文创</t>
+          <t xml:space="preserve">29 桥西文创园</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1708,23 +1688,23 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河文创</t>
+          <t xml:space="preserve">桥西文创园</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="F31" s="2">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="G31" s="2">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 香积寺晨市</t>
+          <t xml:space="preserve">30 杭城事件</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -1744,12 +1724,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">香积寺晨市</t>
+          <t xml:space="preserve">杭城事件</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1769,12 +1749,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">45 钱塘会展中心</t>
+          <t xml:space="preserve">2 断桥文旅</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1784,42 +1764,38 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士</t>
+          <t xml:space="preserve">滨江数创园</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F33" s="2">
+        <v>270</v>
+      </c>
+      <c r="G33" s="2">
+        <v>76</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">33 桥西文创园</t>
+          <t xml:space="preserve">32 大运河艺术馆</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1829,42 +1805,38 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河事件</t>
+          <t xml:space="preserve">大运河艺术馆</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">生态文体</t>
+        </is>
+      </c>
+      <c r="F34" s="2">
+        <v>220</v>
+      </c>
+      <c r="G34" s="2">
+        <v>58</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 杭城事件</t>
+          <t xml:space="preserve">33 钱江新城</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1874,38 +1846,42 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西文创园</t>
+          <t xml:space="preserve">钱江新城</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
-        </is>
-      </c>
-      <c r="F35" s="2">
-        <v>210</v>
-      </c>
-      <c r="G35" s="2">
-        <v>56</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">34 拱宸桥码头</t>
+          <t xml:space="preserve">34 文三数字街</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1915,42 +1891,38 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">拱宸桥码头</t>
+          <t xml:space="preserve">文三数字街</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F36" s="2">
+        <v>240</v>
+      </c>
+      <c r="G36" s="2">
+        <v>66</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">36 西湖接驳</t>
+          <t xml:space="preserve">35 项目验收</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1960,17 +1932,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市路线</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河灯会</t>
+          <t xml:space="preserve">项目验收</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1990,574 +1962,17 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 良渚陶艺村</t>
+          <t xml:space="preserve">17 云栖工坊</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2">
-        <v>36</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水上巴士内环</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">城市路线</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">西湖接驳</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 断桥文旅</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2">
-        <v>37</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">城市路线</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">市民中心站</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">38 滨江数创园</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2">
-        <v>38</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">滨江数创园</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F40" s="2">
-        <v>270</v>
-      </c>
-      <c r="G40" s="2">
-        <v>76</v>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">48 大运河艺术馆</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2">
-        <v>39</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">城市事件</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">钱江新城</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">41 文三数字街</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2">
-        <v>40</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">城市路线</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">44 未来科技城</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2">
-        <v>41</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">文三数字街</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F43" s="2">
-        <v>240</v>
-      </c>
-      <c r="G43" s="2">
-        <v>66</v>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40 地铁快线</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2">
-        <v>42</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外环</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">道具补给</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁补给站</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">27 道具补给站</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2">
-        <v>43</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外环</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">未来路演厅</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F45" s="2">
-        <v>280</v>
-      </c>
-      <c r="G45" s="2">
-        <v>82</v>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">25 杭城事件</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2">
-        <v>44</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">城市路线</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">未来科技城</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17 城市公投</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">路线与岔路节点；经过序号 0 时领取当期经营收入</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2">
-        <v>45</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">水上巴士内环</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">钱塘会展中心</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">钱塘发展</t>
-        </is>
-      </c>
-      <c r="F47" s="2">
-        <v>280</v>
-      </c>
-      <c r="G47" s="2">
-        <v>78</v>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31 水上巴士</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2">
-        <v>46</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外环</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">运河运动公园</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">生态文体</t>
-        </is>
-      </c>
-      <c r="F48" s="2">
-        <v>230</v>
-      </c>
-      <c r="G48" s="2">
-        <v>62</v>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9 钱塘潮</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2">
-        <v>47</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">外环</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">滨江国际社区</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">钱塘发展</t>
-        </is>
-      </c>
-      <c r="F49" s="2">
-        <v>270</v>
-      </c>
-      <c r="G49" s="2">
-        <v>74</v>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 河坊街铺</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2">
-        <v>48</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">地铁快线内环</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">可投资项目</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">大运河艺术馆</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">生态文体</t>
-        </is>
-      </c>
-      <c r="F50" s="2">
-        <v>220</v>
-      </c>
-      <c r="G50" s="2">
-        <v>58</v>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39 钱江新城</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I50"/>
+  <autoFilter ref="A1:I37"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -2663,10 +2078,10 @@
         <v>28</v>
       </c>
       <c r="G2" s="2">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I2" s="2">
         <v>30</v>
@@ -2704,13 +2119,13 @@
         <v>34</v>
       </c>
       <c r="G3" s="2">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H3" s="2">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="I3" s="2">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J3" s="2">
         <v>63</v>
@@ -2722,7 +2137,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">钱塘发展</t>
         </is>
       </c>
       <c r="B4" s="2">
@@ -2730,7 +2145,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">河坊街铺</t>
+          <t xml:space="preserve">滨江国际社区</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2739,25 +2154,25 @@
         </is>
       </c>
       <c r="E4" s="2">
-        <v>150</v>
+        <v>270</v>
       </c>
       <c r="F4" s="2">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="G4" s="2">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="H4" s="2">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I4" s="2">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="J4" s="2">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="K4" s="2">
-        <v>105</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5">
@@ -2767,11 +2182,11 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">南宋食坊</t>
+          <t xml:space="preserve">河坊街铺</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2780,39 +2195,39 @@
         </is>
       </c>
       <c r="E5" s="2">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="F5" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G5" s="2">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="H5" s="2">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="I5" s="2">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J5" s="2">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="K5" s="2">
-        <v>119</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">大莲花场馆</t>
+          <t xml:space="preserve">南宋食坊</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2821,25 +2236,25 @@
         </is>
       </c>
       <c r="E6" s="2">
-        <v>240</v>
+        <v>170</v>
       </c>
       <c r="F6" s="2">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="H6" s="2">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="I6" s="2">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="J6" s="2">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="K6" s="2">
-        <v>168</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7">
@@ -2849,11 +2264,11 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市阳台</t>
+          <t xml:space="preserve">大莲花场馆</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2862,25 +2277,25 @@
         </is>
       </c>
       <c r="E7" s="2">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="F7" s="2">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G7" s="2">
+        <v>92</v>
+      </c>
+      <c r="H7" s="2">
+        <v>119</v>
+      </c>
+      <c r="I7" s="2">
+        <v>70</v>
+      </c>
+      <c r="J7" s="2">
         <v>108</v>
       </c>
-      <c r="H7" s="2">
-        <v>144</v>
-      </c>
-      <c r="I7" s="2">
-        <v>78</v>
-      </c>
-      <c r="J7" s="2">
-        <v>117</v>
-      </c>
       <c r="K7" s="2">
-        <v>182</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8">
@@ -2890,11 +2305,11 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱江创意港</t>
+          <t xml:space="preserve">城市阳台</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2903,39 +2318,39 @@
         </is>
       </c>
       <c r="E8" s="2">
-        <v>230</v>
+        <v>260</v>
       </c>
       <c r="F8" s="2">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G8" s="2">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="H8" s="2">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="I8" s="2">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="J8" s="2">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="K8" s="2">
-        <v>161</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">未来创业营</t>
+          <t xml:space="preserve">运河运动公园</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2944,39 +2359,39 @@
         </is>
       </c>
       <c r="E9" s="2">
-        <v>300</v>
+        <v>230</v>
       </c>
       <c r="F9" s="2">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="G9" s="2">
-        <v>135</v>
+        <v>87</v>
       </c>
       <c r="H9" s="2">
-        <v>180</v>
+        <v>112</v>
       </c>
       <c r="I9" s="2">
-        <v>97</v>
+        <v>66</v>
       </c>
       <c r="J9" s="2">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="K9" s="2">
-        <v>210</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">钱塘发展</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">良渚文创园</t>
+          <t xml:space="preserve">钱江创意港</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -2985,39 +2400,39 @@
         </is>
       </c>
       <c r="E10" s="2">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="F10" s="2">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2">
         <v>87</v>
       </c>
       <c r="H10" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I10" s="2">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J10" s="2">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="K10" s="2">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">良渚陶艺村</t>
+          <t xml:space="preserve">未来创业营</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3026,39 +2441,39 @@
         </is>
       </c>
       <c r="E11" s="2">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="F11" s="2">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="G11" s="2">
-        <v>87</v>
+        <v>126</v>
       </c>
       <c r="H11" s="2">
-        <v>116</v>
+        <v>162</v>
       </c>
       <c r="I11" s="2">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="J11" s="2">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="K11" s="2">
-        <v>154</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">云栖工坊</t>
+          <t xml:space="preserve">良渚文创园</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3067,25 +2482,25 @@
         </is>
       </c>
       <c r="E12" s="2">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="F12" s="2">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G12" s="2">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="H12" s="2">
-        <v>136</v>
+        <v>104</v>
       </c>
       <c r="I12" s="2">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="J12" s="2">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="K12" s="2">
-        <v>175</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13">
@@ -3095,11 +2510,11 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">西溪营地</t>
+          <t xml:space="preserve">良渚陶艺村</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3108,39 +2523,39 @@
         </is>
       </c>
       <c r="E13" s="2">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="F13" s="2">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G13" s="2">
         <v>81</v>
       </c>
       <c r="H13" s="2">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I13" s="2">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="J13" s="2">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K13" s="2">
-        <v>147</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="B14" s="2">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河夜游</t>
+          <t xml:space="preserve">云栖工坊</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3149,39 +2564,39 @@
         </is>
       </c>
       <c r="E14" s="2">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F14" s="2">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="H14" s="2">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="I14" s="2">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="J14" s="2">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="K14" s="2">
-        <v>140</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">武林夜市</t>
+          <t xml:space="preserve">西溪营地</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -3190,39 +2605,39 @@
         </is>
       </c>
       <c r="E15" s="2">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="F15" s="2">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G15" s="2">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H15" s="2">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I15" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J15" s="2">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="K15" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="B16" s="2">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">小河市集</t>
+          <t xml:space="preserve">运河夜游</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -3231,25 +2646,25 @@
         </is>
       </c>
       <c r="E16" s="2">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="F16" s="2">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G16" s="2">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H16" s="2">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I16" s="2">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J16" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="K16" s="2">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17">
@@ -3259,11 +2674,11 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西生活馆</t>
+          <t xml:space="preserve">武林夜市</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -3272,224 +2687,224 @@
         </is>
       </c>
       <c r="E17" s="2">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="F17" s="2">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G17" s="2">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H17" s="2">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I17" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J17" s="2">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="K17" s="2">
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河文创</t>
+          <t xml:space="preserve">小河市集</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E18" s="2">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="F18" s="2">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G18" s="2">
+        <v>64</v>
+      </c>
+      <c r="H18" s="2">
+        <v>83</v>
+      </c>
+      <c r="I18" s="2">
+        <v>49</v>
+      </c>
+      <c r="J18" s="2">
         <v>81</v>
       </c>
-      <c r="H18" s="2">
-        <v>108</v>
-      </c>
-      <c r="I18" s="2">
-        <v>58</v>
-      </c>
-      <c r="J18" s="2">
-        <v>90</v>
-      </c>
       <c r="K18" s="2">
-        <v>140</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西文创园</t>
+          <t xml:space="preserve">未来路演厅</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E19" s="2">
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="F19" s="2">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="G19" s="2">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="H19" s="2">
-        <v>112</v>
+        <v>148</v>
       </c>
       <c r="I19" s="2">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="J19" s="2">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="K19" s="2">
-        <v>147</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">滨江数创园</t>
+          <t xml:space="preserve">桥西生活馆</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E20" s="2">
-        <v>270</v>
+        <v>190</v>
       </c>
       <c r="F20" s="2">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="G20" s="2">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="H20" s="2">
-        <v>152</v>
+        <v>90</v>
       </c>
       <c r="I20" s="2">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="J20" s="2">
-        <v>122</v>
+        <v>86</v>
       </c>
       <c r="K20" s="2">
-        <v>189</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文三数字街</t>
+          <t xml:space="preserve">运河文创</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">水上巴士内环</t>
         </is>
       </c>
       <c r="E21" s="2">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="F21" s="2">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="G21" s="2">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="H21" s="2">
-        <v>132</v>
+        <v>97</v>
       </c>
       <c r="I21" s="2">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="J21" s="2">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="K21" s="2">
-        <v>168</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">钱塘发展</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">未来路演厅</t>
+          <t xml:space="preserve">钱塘会展中心</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">水上巴士内环</t>
         </is>
       </c>
       <c r="E22" s="2">
         <v>280</v>
       </c>
       <c r="F22" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G22" s="2">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="H22" s="2">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="I22" s="2">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="J22" s="2">
         <v>126</v>
@@ -3501,15 +2916,15 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘会展中心</t>
+          <t xml:space="preserve">桥西文创园</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3518,121 +2933,121 @@
         </is>
       </c>
       <c r="E23" s="2">
-        <v>280</v>
+        <v>210</v>
       </c>
       <c r="F23" s="2">
+        <v>56</v>
+      </c>
+      <c r="G23" s="2">
         <v>78</v>
       </c>
-      <c r="G23" s="2">
-        <v>117</v>
-      </c>
       <c r="H23" s="2">
-        <v>156</v>
+        <v>101</v>
       </c>
       <c r="I23" s="2">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="J23" s="2">
-        <v>126</v>
+        <v>95</v>
       </c>
       <c r="K23" s="2">
-        <v>196</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="B24" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河运动公园</t>
+          <t xml:space="preserve">滨江数创园</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="E24" s="2">
-        <v>230</v>
+        <v>270</v>
       </c>
       <c r="F24" s="2">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="G24" s="2">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="H24" s="2">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="I24" s="2">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="J24" s="2">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="K24" s="2">
-        <v>161</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="B25" s="2">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">滨江国际社区</t>
+          <t xml:space="preserve">大运河艺术馆</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="E25" s="2">
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="F25" s="2">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="G25" s="2">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="H25" s="2">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="I25" s="2">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="J25" s="2">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="K25" s="2">
-        <v>189</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="B26" s="2">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">大运河艺术馆</t>
+          <t xml:space="preserve">文三数字街</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -3641,25 +3056,25 @@
         </is>
       </c>
       <c r="E26" s="2">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="F26" s="2">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G26" s="2">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H26" s="2">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I26" s="2">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="J26" s="2">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="K26" s="2">
-        <v>154</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -3784,12 +3199,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">分红 +8%</t>
+          <t xml:space="preserve">分红 +6%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">该板块所有参与项目的到访分红 ×1.08</t>
+          <t xml:space="preserve">该板块所有参与项目的到访分红 ×1.06</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -4366,7 +3781,7 @@
         </is>
       </c>
       <c r="C7" s="2">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -4391,7 +3806,7 @@
         </is>
       </c>
       <c r="C8" s="2">
-        <v>220</v>
+        <v>260</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -4416,7 +3831,7 @@
         </is>
       </c>
       <c r="C9" s="2">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4299,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1650/1725/1800/1875</t>
+          <t xml:space="preserve">1880/1980/2180/2230</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -4987,7 +4402,7 @@
         </is>
       </c>
       <c r="C8" s="2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -5007,7 +4422,7 @@
         </is>
       </c>
       <c r="C9" s="2">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -5199,7 +4614,7 @@
         </is>
       </c>
       <c r="C18" s="2">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: enlarge board art and separate project labels
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M4原型.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M4原型.xlsx
@@ -950,7 +950,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 外环·钱塘线 / 31 地铁快线</t>
+          <t xml:space="preserve">12 外环·钱塘线 / 32 地铁快线</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 良渚文创园</t>
+          <t xml:space="preserve">15 项目验收</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1097,33 +1097,37 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">良渚文创园</t>
+          <t xml:space="preserve">项目验收</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
-        </is>
-      </c>
-      <c r="F17" s="2">
-        <v>220</v>
-      </c>
-      <c r="G17" s="2">
-        <v>58</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 良渚陶艺村</t>
+          <t xml:space="preserve">16 良渚文创园</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1143,12 +1147,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">良渚陶艺村</t>
+          <t xml:space="preserve">良渚文创园</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="F18" s="2">
@@ -1159,7 +1163,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">17 云栖工坊</t>
+          <t xml:space="preserve">17 良渚陶艺村</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1184,23 +1188,23 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">云栖工坊</t>
+          <t xml:space="preserve">良渚陶艺村</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F19" s="2">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="G19" s="2">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">18 人才事件</t>
+          <t xml:space="preserve">18 云栖工坊</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1220,37 +1224,33 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">人才事件</t>
+          <t xml:space="preserve">云栖工坊</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F20" s="2">
+        <v>250</v>
+      </c>
+      <c r="G20" s="2">
+        <v>68</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">19 西溪营地</t>
+          <t xml:space="preserve">19 人才事件</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1265,33 +1265,37 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">西溪营地</t>
+          <t xml:space="preserve">人才事件</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
-        </is>
-      </c>
-      <c r="F21" s="2">
-        <v>210</v>
-      </c>
-      <c r="G21" s="2">
-        <v>54</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20 运河夜游</t>
+          <t xml:space="preserve">20 西溪营地</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1311,23 +1315,23 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河夜游</t>
+          <t xml:space="preserve">西溪营地</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F22" s="2">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="G22" s="2">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">21 外环·运河线 / 27 水上巴士线</t>
+          <t xml:space="preserve">21 运河夜游</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1352,12 +1356,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">武林夜市</t>
+          <t xml:space="preserve">运河夜游</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="F23" s="2">
@@ -1368,7 +1372,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 小河市集</t>
+          <t xml:space="preserve">22 外环·运河线 / 28 水上巴士线</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1393,7 +1397,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">小河市集</t>
+          <t xml:space="preserve">武林夜市</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1402,14 +1406,14 @@
         </is>
       </c>
       <c r="F24" s="2">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="G24" s="2">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">23 未来路演厅</t>
+          <t xml:space="preserve">23 小河市集</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1434,23 +1438,23 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">未来路演厅</t>
+          <t xml:space="preserve">小河市集</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="F25" s="2">
-        <v>280</v>
+        <v>180</v>
       </c>
       <c r="G25" s="2">
-        <v>82</v>
+        <v>46</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">24 桥西生活馆</t>
+          <t xml:space="preserve">24 未来路演厅</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1475,23 +1479,23 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西生活馆</t>
+          <t xml:space="preserve">未来路演厅</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="F26" s="2">
-        <v>190</v>
+        <v>280</v>
       </c>
       <c r="G26" s="2">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25 地铁补给站</t>
+          <t xml:space="preserve">25 桥西生活馆</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1511,37 +1515,33 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁补给站</t>
+          <t xml:space="preserve">桥西生活馆</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">城市生活</t>
+        </is>
+      </c>
+      <c r="F27" s="2">
+        <v>190</v>
+      </c>
+      <c r="G27" s="2">
+        <v>50</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">26 道具补给站</t>
+          <t xml:space="preserve">26 地铁补给站</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给站</t>
+          <t xml:space="preserve">地铁补给站</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 我的公寓</t>
+          <t xml:space="preserve">27 道具补给站</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1596,38 +1596,42 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">道具补给</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河文创</t>
+          <t xml:space="preserve">道具补给站</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
-        </is>
-      </c>
-      <c r="F29" s="2">
-        <v>200</v>
-      </c>
-      <c r="G29" s="2">
-        <v>54</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">28 钱塘会展中心</t>
+          <t xml:space="preserve">0 我的公寓</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
         </is>
       </c>
     </row>
@@ -1647,23 +1651,23 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘会展中心</t>
+          <t xml:space="preserve">运河文创</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F30" s="2">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="G30" s="2">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">29 桥西文创园</t>
+          <t xml:space="preserve">29 钱塘会展中心</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1688,23 +1692,23 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西文创园</t>
+          <t xml:space="preserve">钱塘会展中心</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">钱塘发展</t>
         </is>
       </c>
       <c r="F31" s="2">
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="G31" s="2">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 杭城事件</t>
+          <t xml:space="preserve">30 桥西文创园</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -1724,37 +1728,33 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭城事件</t>
+          <t xml:space="preserve">桥西文创园</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">文旅消费</t>
+        </is>
+      </c>
+      <c r="F32" s="2">
+        <v>210</v>
+      </c>
+      <c r="G32" s="2">
+        <v>56</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 断桥文旅</t>
+          <t xml:space="preserve">31 杭城事件</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1764,38 +1764,42 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">水上巴士内环</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">滨江数创园</t>
+          <t xml:space="preserve">杭城事件</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F33" s="2">
-        <v>270</v>
-      </c>
-      <c r="G33" s="2">
-        <v>76</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">32 大运河艺术馆</t>
+          <t xml:space="preserve">2 断桥文旅</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1815,23 +1819,23 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">大运河艺术馆</t>
+          <t xml:space="preserve">滨江数创园</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="F34" s="2">
-        <v>220</v>
+        <v>270</v>
       </c>
       <c r="G34" s="2">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">33 钱江新城</t>
+          <t xml:space="preserve">33 大运河艺术馆</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -1851,37 +1855,33 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱江新城</t>
+          <t xml:space="preserve">大运河艺术馆</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">生态文体</t>
+        </is>
+      </c>
+      <c r="F35" s="2">
+        <v>220</v>
+      </c>
+      <c r="G35" s="2">
+        <v>58</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">34 文三数字街</t>
+          <t xml:space="preserve">34 钱江新城</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1896,33 +1896,37 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文三数字街</t>
+          <t xml:space="preserve">钱江新城</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F36" s="2">
-        <v>240</v>
-      </c>
-      <c r="G36" s="2">
-        <v>66</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35 项目验收</t>
+          <t xml:space="preserve">35 文三数字街</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1937,37 +1941,33 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">项目验收</t>
+          <t xml:space="preserve">文三数字街</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F37" s="2">
+        <v>240</v>
+      </c>
+      <c r="G37" s="2">
+        <v>66</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">17 云栖工坊</t>
+          <t xml:space="preserve">16 良渚文创园</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="B26" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: integrate larger icons into board cards
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M4原型.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M4原型.xlsx
@@ -782,7 +782,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 杭城事件</t>
+          <t xml:space="preserve">8 大莲花场馆</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -802,37 +802,33 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭城事件</t>
+          <t xml:space="preserve">大莲花场馆</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">钱塘发展</t>
+        </is>
+      </c>
+      <c r="F10" s="2">
+        <v>240</v>
+      </c>
+      <c r="G10" s="2">
+        <v>66</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9 大莲花场馆</t>
+          <t xml:space="preserve">9 城市阳台</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -852,7 +848,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">大莲花场馆</t>
+          <t xml:space="preserve">城市阳台</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -861,14 +857,14 @@
         </is>
       </c>
       <c r="F11" s="2">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="G11" s="2">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10 城市阳台</t>
+          <t xml:space="preserve">10 运河运动公园</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -893,23 +889,23 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市阳台</t>
+          <t xml:space="preserve">运河运动公园</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F12" s="2">
-        <v>260</v>
+        <v>230</v>
       </c>
       <c r="G12" s="2">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 运河运动公园</t>
+          <t xml:space="preserve">11 外环·钱塘线 / 31 地铁快线</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -934,12 +930,12 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河运动公园</t>
+          <t xml:space="preserve">钱江创意港</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">钱塘发展</t>
         </is>
       </c>
       <c r="F13" s="2">
@@ -950,7 +946,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 外环·钱塘线 / 32 地铁快线</t>
+          <t xml:space="preserve">12 创业事件</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -970,33 +966,37 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱江创意港</t>
+          <t xml:space="preserve">创业事件</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
-        </is>
-      </c>
-      <c r="F14" s="2">
-        <v>230</v>
-      </c>
-      <c r="G14" s="2">
-        <v>62</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13 创业事件</t>
+          <t xml:space="preserve">13 未来创业营</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1011,37 +1011,33 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">创业事件</t>
+          <t xml:space="preserve">未来创业营</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F15" s="2">
+        <v>300</v>
+      </c>
+      <c r="G15" s="2">
+        <v>90</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">14 未来创业营</t>
+          <t xml:space="preserve">14 良渚文创园</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1061,23 +1057,23 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">未来创业营</t>
+          <t xml:space="preserve">良渚文创园</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="F16" s="2">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="G16" s="2">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 项目验收</t>
+          <t xml:space="preserve">15 良渚陶艺村</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1097,37 +1093,33 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">项目验收</t>
+          <t xml:space="preserve">良渚陶艺村</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">生态文体</t>
+        </is>
+      </c>
+      <c r="F17" s="2">
+        <v>220</v>
+      </c>
+      <c r="G17" s="2">
+        <v>58</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 良渚文创园</t>
+          <t xml:space="preserve">16 云栖工坊</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1147,23 +1139,23 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">良渚文创园</t>
+          <t xml:space="preserve">云栖工坊</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="F18" s="2">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="G18" s="2">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">17 良渚陶艺村</t>
+          <t xml:space="preserve">17 人才事件</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1183,33 +1175,37 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">良渚陶艺村</t>
+          <t xml:space="preserve">人才事件</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
-        </is>
-      </c>
-      <c r="F19" s="2">
-        <v>220</v>
-      </c>
-      <c r="G19" s="2">
-        <v>58</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">18 云栖工坊</t>
+          <t xml:space="preserve">18 西溪营地</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1229,23 +1225,23 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">云栖工坊</t>
+          <t xml:space="preserve">西溪营地</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F20" s="2">
-        <v>250</v>
+        <v>210</v>
       </c>
       <c r="G20" s="2">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">19 人才事件</t>
+          <t xml:space="preserve">19 运河夜游</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1265,37 +1261,33 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">人才事件</t>
+          <t xml:space="preserve">运河夜游</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">文旅消费</t>
+        </is>
+      </c>
+      <c r="F21" s="2">
+        <v>200</v>
+      </c>
+      <c r="G21" s="2">
+        <v>52</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20 西溪营地</t>
+          <t xml:space="preserve">20 外环·运河线 / 26 水上巴士线</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1315,23 +1307,23 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">西溪营地</t>
+          <t xml:space="preserve">武林夜市</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="F22" s="2">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="G22" s="2">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">21 运河夜游</t>
+          <t xml:space="preserve">21 小河市集</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1356,23 +1348,23 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河夜游</t>
+          <t xml:space="preserve">小河市集</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
+          <t xml:space="preserve">城市生活</t>
         </is>
       </c>
       <c r="F23" s="2">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="G23" s="2">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 外环·运河线 / 28 水上巴士线</t>
+          <t xml:space="preserve">22 未来路演厅</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1397,23 +1389,23 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">武林夜市</t>
+          <t xml:space="preserve">未来路演厅</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
+          <t xml:space="preserve">数字科技</t>
         </is>
       </c>
       <c r="F24" s="2">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="G24" s="2">
-        <v>52</v>
+        <v>82</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">23 小河市集</t>
+          <t xml:space="preserve">23 桥西生活馆</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1438,7 +1430,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">小河市集</t>
+          <t xml:space="preserve">桥西生活馆</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1447,14 +1439,14 @@
         </is>
       </c>
       <c r="F25" s="2">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="G25" s="2">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">24 未来路演厅</t>
+          <t xml:space="preserve">24 地铁补给站</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1474,33 +1466,37 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">道具补给</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">未来路演厅</t>
+          <t xml:space="preserve">地铁补给站</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F26" s="2">
-        <v>280</v>
-      </c>
-      <c r="G26" s="2">
-        <v>82</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25 桥西生活馆</t>
+          <t xml:space="preserve">25 道具补给站</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
         </is>
       </c>
     </row>
@@ -1515,33 +1511,37 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">道具补给</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西生活馆</t>
+          <t xml:space="preserve">道具补给站</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市生活</t>
-        </is>
-      </c>
-      <c r="F27" s="2">
-        <v>190</v>
-      </c>
-      <c r="G27" s="2">
-        <v>50</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">26 地铁补给站</t>
+          <t xml:space="preserve">0 我的公寓</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
         </is>
       </c>
     </row>
@@ -1551,42 +1551,38 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">水上巴士内环</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁补给站</t>
+          <t xml:space="preserve">运河文创</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">生态文体</t>
+        </is>
+      </c>
+      <c r="F28" s="2">
+        <v>200</v>
+      </c>
+      <c r="G28" s="2">
+        <v>54</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">27 道具补给站</t>
+          <t xml:space="preserve">27 钱塘会展中心</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1596,42 +1592,38 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">水上巴士内环</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">道具补给站</t>
+          <t xml:space="preserve">钱塘会展中心</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">钱塘发展</t>
+        </is>
+      </c>
+      <c r="F29" s="2">
+        <v>280</v>
+      </c>
+      <c r="G29" s="2">
+        <v>78</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 我的公寓</t>
+          <t xml:space="preserve">28 桥西文创园</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率获得 1 张道具；持有满 3 张时兑换 60 金币</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1651,23 +1643,23 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">运河文创</t>
+          <t xml:space="preserve">桥西文创园</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
+          <t xml:space="preserve">文旅消费</t>
         </is>
       </c>
       <c r="F30" s="2">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="G30" s="2">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">29 钱塘会展中心</t>
+          <t xml:space="preserve">29 杭城事件</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1687,33 +1679,37 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘会展中心</t>
+          <t xml:space="preserve">杭城事件</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱塘发展</t>
-        </is>
-      </c>
-      <c r="F31" s="2">
-        <v>280</v>
-      </c>
-      <c r="G31" s="2">
-        <v>78</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 桥西文创园</t>
+          <t xml:space="preserve">30 杭城事件</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1728,33 +1724,37 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">桥西文创园</t>
+          <t xml:space="preserve">杭城事件</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文旅消费</t>
-        </is>
-      </c>
-      <c r="F32" s="2">
-        <v>210</v>
-      </c>
-      <c r="G32" s="2">
-        <v>56</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">31 杭城事件</t>
+          <t xml:space="preserve">2 断桥文旅</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1764,42 +1764,38 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">杭城事件</t>
+          <t xml:space="preserve">滨江数创园</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F33" s="2">
+        <v>270</v>
+      </c>
+      <c r="G33" s="2">
+        <v>76</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 断桥文旅</t>
+          <t xml:space="preserve">32 大运河艺术馆</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1819,23 +1815,23 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">滨江数创园</t>
+          <t xml:space="preserve">大运河艺术馆</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
+          <t xml:space="preserve">生态文体</t>
         </is>
       </c>
       <c r="F34" s="2">
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="G34" s="2">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">33 大运河艺术馆</t>
+          <t xml:space="preserve">33 钱江新城</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -1855,33 +1851,37 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">大运河艺术馆</t>
+          <t xml:space="preserve">钱江新城</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">生态文体</t>
-        </is>
-      </c>
-      <c r="F35" s="2">
-        <v>220</v>
-      </c>
-      <c r="G35" s="2">
-        <v>58</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">34 钱江新城</t>
+          <t xml:space="preserve">34 文三数字街</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -1896,37 +1896,33 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">城市事件</t>
+          <t xml:space="preserve">可投资项目</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">钱江新城</t>
+          <t xml:space="preserve">文三数字街</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">数字科技</t>
+        </is>
+      </c>
+      <c r="F36" s="2">
+        <v>240</v>
+      </c>
+      <c r="G36" s="2">
+        <v>66</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35 文三数字街</t>
+          <t xml:space="preserve">35 项目验收</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
+          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
         </is>
       </c>
     </row>
@@ -1941,33 +1937,37 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可投资项目</t>
+          <t xml:space="preserve">城市事件</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文三数字街</t>
+          <t xml:space="preserve">项目验收</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">数字科技</t>
-        </is>
-      </c>
-      <c r="F37" s="2">
-        <v>240</v>
-      </c>
-      <c r="G37" s="2">
-        <v>66</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 良渚文创园</t>
+          <t xml:space="preserve">14 良渚文创园</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">无主时可独资或五五合伙投资；到访他人项目时支付分红</t>
+          <t xml:space="preserve">等概率触发 1 个城市事件；只影响现金、道具或行动状态</t>
         </is>
       </c>
     </row>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -2346,7 +2346,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="B26" s="2">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>

</xml_diff>